<commit_message>
chore(hmb): remove candidatos que desistiram da vaga (Milton e Marcos)
Conforme email da supervisao (19/08/2026):

Retirados (desistiram da vaga):
- Milton Gustavo Sabino Costa (Aux. de Eletricista, folguista diurno provisorio)
- Marcos Vinicius de Lira (Eletricista, folguista diurno provisorio)

Mikael da Rocha (Tecnico de Climatizacao) tambem foi citado no email como
desistente, mas nao foi encontrado na planilha em nenhuma linha/grafia — nunca
chegou a ser adicionado a automacao, entao nenhuma acao foi necessaria pra ele.

Validado: parser real confirma 22 colaboradores carregados (era 24), com
Milton e Marcos ausentes e os demais intactos. 88 testes de backend passando.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/hmb/Escala_HMB_Segunda_Quinzena_Agosto_2026V2.xlsx
+++ b/backend/data/hmb/Escala_HMB_Segunda_Quinzena_Agosto_2026V2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Escala 16-31 Ago" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Times e Folguistas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Premissas e Pendências" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escala 16-31 Ago" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Times e Folguistas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas e Pendências" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Marcos Vinicius de Lira</t>
+          <t>Osmar Silva</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
@@ -1307,12 +1307,12 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>Folguista diurno — provisório ímpar</t>
+          <t>Noturno par — provisório</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>07:00–19:00</t>
+          <t>19:00–07:00</t>
         </is>
       </c>
       <c r="F10" s="17" t="n"/>
@@ -1320,41 +1320,33 @@
       <c r="H10" s="17" t="n"/>
       <c r="I10" s="17" t="n"/>
       <c r="J10" s="17" t="n"/>
-      <c r="K10" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="K10" s="17" t="n"/>
       <c r="L10" s="17" t="n"/>
-      <c r="M10" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N10" s="17" t="n"/>
-      <c r="O10" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P10" s="17" t="n"/>
-      <c r="Q10" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R10" s="17" t="n"/>
-      <c r="S10" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T10" s="17" t="n"/>
-      <c r="U10" s="18" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="M10" s="17" t="n"/>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O10" s="17" t="n"/>
+      <c r="P10" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q10" s="17" t="n"/>
+      <c r="R10" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S10" s="17" t="n"/>
+      <c r="T10" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U10" s="18" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -1364,7 +1356,7 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Osmar Silva</t>
+          <t>Caio Pereira</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
@@ -1374,21 +1366,29 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>Noturno par — provisório</t>
+          <t>Folguista volante — provisório diurno par</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>19:00–07:00</t>
+          <t>07:00–19:00</t>
         </is>
       </c>
       <c r="F11" s="17" t="n"/>
       <c r="G11" s="17" t="n"/>
       <c r="H11" s="17" t="n"/>
       <c r="I11" s="17" t="n"/>
-      <c r="J11" s="17" t="n"/>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="K11" s="17" t="n"/>
-      <c r="L11" s="17" t="n"/>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="M11" s="17" t="n"/>
       <c r="N11" s="17" t="inlineStr">
         <is>
@@ -1416,142 +1416,146 @@
       <c r="U11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>Caio Pereira</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Eletricista</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>Folguista volante — provisório diurno par</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>AUX. ELÉTRICA</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Ronaldo Manoel dos Santos</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>Aux. de Eletricista</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Diurno par — provisório</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>07:00–19:00</t>
         </is>
       </c>
-      <c r="F12" s="17" t="n"/>
-      <c r="G12" s="17" t="n"/>
-      <c r="H12" s="17" t="n"/>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K12" s="17" t="n"/>
-      <c r="L12" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M12" s="17" t="n"/>
-      <c r="N12" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O12" s="17" t="n"/>
-      <c r="P12" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q12" s="17" t="n"/>
-      <c r="R12" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S12" s="17" t="n"/>
-      <c r="T12" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U12" s="18" t="n"/>
+      <c r="F12" s="22" t="n"/>
+      <c r="G12" s="22" t="n"/>
+      <c r="H12" s="22" t="n"/>
+      <c r="I12" s="22" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K12" s="22" t="n"/>
+      <c r="L12" s="22" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M12" s="22" t="n"/>
+      <c r="N12" s="22" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O12" s="22" t="n"/>
+      <c r="P12" s="22" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q12" s="22" t="n"/>
+      <c r="R12" s="22" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S12" s="22" t="n"/>
+      <c r="T12" s="22" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U12" s="22" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>AUX. ELÉTRICA</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>Ronaldo Manoel dos Santos</t>
-        </is>
-      </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Jeferson Souza da Silva</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Aux. de Eletricista</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>Diurno par — provisório</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Diurno ímpar</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>07:00–19:00</t>
         </is>
       </c>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="22" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="J13" s="22" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K13" s="22" t="n"/>
-      <c r="L13" s="22" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M13" s="22" t="n"/>
-      <c r="N13" s="22" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O13" s="22" t="n"/>
-      <c r="P13" s="22" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q13" s="22" t="n"/>
-      <c r="R13" s="22" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S13" s="22" t="n"/>
-      <c r="T13" s="22" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U13" s="22" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="n"/>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="n"/>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="n"/>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="n"/>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="n"/>
+      <c r="S13" s="8" t="n"/>
+      <c r="T13" s="8" t="n"/>
+      <c r="U13" s="9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1561,7 +1565,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Jeferson Souza da Silva</t>
+          <t>Lucas Henrique Martins</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -1571,125 +1575,129 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Diurno ímpar</t>
+          <t>Noturno par</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>07:00–19:00</t>
+          <t>19:00–07:00</t>
         </is>
       </c>
       <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="n"/>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="n"/>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="n"/>
-      <c r="M14" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N14" s="8" t="n"/>
-      <c r="O14" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P14" s="8" t="n"/>
-      <c r="Q14" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R14" s="8" t="n"/>
+      <c r="M14" s="8" t="n"/>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="n"/>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="n"/>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="S14" s="8" t="n"/>
-      <c r="T14" s="8" t="n"/>
-      <c r="U14" s="9" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="T14" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>AUX. ELÉTRICA</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Lucas Henrique Martins</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Em processo de contratação</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Aux. de Eletricista</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Noturno par</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Noturno ímpar</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>19:00–07:00</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="n"/>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="n"/>
-      <c r="L15" s="8" t="n"/>
-      <c r="M15" s="8" t="n"/>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="n"/>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q15" s="8" t="n"/>
-      <c r="R15" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S15" s="8" t="n"/>
-      <c r="T15" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U15" s="9" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="n"/>
+      <c r="M15" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="N15" s="12" t="n"/>
+      <c r="O15" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="P15" s="12" t="n"/>
+      <c r="Q15" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="R15" s="12" t="n"/>
+      <c r="S15" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="T15" s="12" t="n"/>
+      <c r="U15" s="13" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1709,7 +1717,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Noturno ímpar</t>
+          <t>Folguista noturno</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -1717,275 +1725,267 @@
           <t>19:00–07:00</t>
         </is>
       </c>
-      <c r="F16" s="12" t="n"/>
-      <c r="G16" s="12" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H16" s="12" t="n"/>
-      <c r="I16" s="12" t="inlineStr">
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n"/>
-      <c r="K16" s="12" t="inlineStr">
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="L16" s="12" t="n"/>
-      <c r="M16" s="12" t="inlineStr">
+      <c r="K16" s="12" t="n"/>
+      <c r="L16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="N16" s="12" t="n"/>
-      <c r="O16" s="12" t="inlineStr">
+      <c r="M16" s="12" t="n"/>
+      <c r="N16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="P16" s="12" t="n"/>
-      <c r="Q16" s="12" t="inlineStr">
+      <c r="O16" s="12" t="n"/>
+      <c r="P16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="R16" s="12" t="n"/>
-      <c r="S16" s="12" t="inlineStr">
+      <c r="Q16" s="12" t="n"/>
+      <c r="R16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="T16" s="12" t="n"/>
-      <c r="U16" s="13" t="inlineStr">
+      <c r="S16" s="12" t="n"/>
+      <c r="T16" s="12" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
+      <c r="U16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>AUX. ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>Milton Gustavo Sabino Costa</t>
-        </is>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>Aux. de Eletricista</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
-        <is>
-          <t>Folguista diurno — provisório ímpar</t>
-        </is>
-      </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Carlos Alberto Bomfim</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Técnico de Climatização</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Diurno par</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>07:00–19:00</t>
         </is>
       </c>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="17" t="n"/>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="17" t="n"/>
-      <c r="J17" s="17" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L17" s="17" t="n"/>
-      <c r="M17" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N17" s="17" t="n"/>
-      <c r="O17" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P17" s="17" t="n"/>
-      <c r="Q17" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R17" s="17" t="n"/>
-      <c r="S17" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T17" s="17" t="n"/>
-      <c r="U17" s="18" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>AUX. ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>Em processo de contratação</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Aux. de Eletricista</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>Folguista noturno</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Douglas Rodrigues</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Técnico de Climatização</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Diurno ímpar</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>07:00–19:00</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="n"/>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="n"/>
+      <c r="K18" s="8" t="n"/>
+      <c r="L18" s="8" t="n"/>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="n"/>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P18" s="8" t="n"/>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="R18" s="8" t="n"/>
+      <c r="S18" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T18" s="8" t="n"/>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Gabriel Passareni Trindade Silva</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Técnico de Climatização</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Noturno par</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>19:00–07:00</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="n"/>
-      <c r="J18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="K18" s="12" t="n"/>
-      <c r="L18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="M18" s="12" t="n"/>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="O18" s="12" t="n"/>
-      <c r="P18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="Q18" s="12" t="n"/>
-      <c r="R18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="S18" s="12" t="n"/>
-      <c r="T18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="U18" s="13" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Carlos Alberto Bomfim</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Técnico de Climatização</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Diurno par</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>07:00–19:00</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="n"/>
-      <c r="N19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="n"/>
-      <c r="P19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q19" s="5" t="n"/>
-      <c r="R19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S19" s="5" t="n"/>
-      <c r="T19" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U19" s="5" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="n"/>
+      <c r="L19" s="8" t="n"/>
+      <c r="M19" s="8" t="n"/>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="n"/>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q19" s="8" t="n"/>
+      <c r="R19" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S19" s="8" t="n"/>
+      <c r="T19" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Douglas Rodrigues</t>
+          <t>Lesle Venini Izidoro dos Santos</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Diurno ímpar</t>
+          <t>Noturno ímpar</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>07:00–19:00</t>
+          <t>19:00–07:00</t>
         </is>
       </c>
       <c r="F20" s="8" t="n"/>
@@ -2026,13 +2026,13 @@
         </is>
       </c>
       <c r="J20" s="8" t="n"/>
-      <c r="K20" s="8" t="n"/>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="L20" s="8" t="n"/>
-      <c r="M20" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="M20" s="8" t="n"/>
       <c r="N20" s="8" t="n"/>
       <c r="O20" s="8" t="inlineStr">
         <is>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Gabriel Passareni Trindade Silva</t>
+          <t>Israel Pereira Bomfim</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -2076,15 +2076,19 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Noturno par</t>
+          <t>Folguista diurno — 12x36 par</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>19:00–07:00</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="n"/>
+          <t>07:00–19:00</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="inlineStr">
         <is>
@@ -2098,7 +2102,11 @@
         </is>
       </c>
       <c r="K21" s="8" t="n"/>
-      <c r="L21" s="8" t="n"/>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="M21" s="8" t="n"/>
       <c r="N21" s="8" t="inlineStr">
         <is>
@@ -2126,355 +2134,355 @@
       <c r="U21" s="9" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>CLIMATIZAÇÃO</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Lesle Venini Izidoro dos Santos</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Claudemir Ribeiro dos Santos</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>Técnico de Climatização</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Folguista diurno — provisório par</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>07:00–19:00</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
+      <c r="H22" s="17" t="n"/>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="n"/>
+      <c r="L22" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="n"/>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O22" s="17" t="n"/>
+      <c r="P22" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q22" s="17" t="n"/>
+      <c r="R22" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S22" s="17" t="n"/>
+      <c r="T22" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U22" s="18" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>AUX. CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Gerson Castro</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Aux. Manutenção / Climatização</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Diurno par</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>07:00–19:00</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="n"/>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="n"/>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="n"/>
+      <c r="L23" s="17" t="n"/>
+      <c r="M23" s="17" t="n"/>
+      <c r="N23" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O23" s="17" t="n"/>
+      <c r="P23" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q23" s="17" t="n"/>
+      <c r="R23" s="17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S23" s="17" t="n"/>
+      <c r="T23" s="17" t="n"/>
+      <c r="U23" s="18" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>AUX. CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Gustavo Rafael Pereira Vargas</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Aux. Manutenção / Climatização</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Diurno ímpar</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>07:00–19:00</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="n"/>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="n"/>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="n"/>
+      <c r="O24" s="5" t="n"/>
+      <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="n"/>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="n"/>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>AUX. CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Victor Hugo Gomes de Araujo</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Aux. Manutenção / Climatização</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Noturno par</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>19:00–07:00</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="n"/>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="n"/>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O25" s="8" t="n"/>
+      <c r="P25" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q25" s="8" t="n"/>
+      <c r="R25" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S25" s="8" t="n"/>
+      <c r="T25" s="8" t="n"/>
+      <c r="U25" s="9" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>AUX. CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Jeferson Leandro Nardy Andrade</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Aux. Manutenção / Climatização</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Noturno ímpar</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>19:00–07:00</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="n"/>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J22" s="8" t="n"/>
-      <c r="K22" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L22" s="8" t="n"/>
-      <c r="M22" s="8" t="n"/>
-      <c r="N22" s="8" t="n"/>
-      <c r="O22" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P22" s="8" t="n"/>
-      <c r="Q22" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R22" s="8" t="n"/>
-      <c r="S22" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T22" s="8" t="n"/>
-      <c r="U22" s="9" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Israel Pereira Bomfim</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Técnico de Climatização</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Folguista diurno — 12x36 par</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>07:00–19:00</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="n"/>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="n"/>
-      <c r="L23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M23" s="8" t="n"/>
-      <c r="N23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O23" s="8" t="n"/>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q23" s="8" t="n"/>
-      <c r="R23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S23" s="8" t="n"/>
-      <c r="T23" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U23" s="9" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>Claudemir Ribeiro dos Santos</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>Técnico de Climatização</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>Folguista diurno — provisório par</t>
-        </is>
-      </c>
-      <c r="E24" s="15" t="inlineStr">
-        <is>
-          <t>07:00–19:00</t>
-        </is>
-      </c>
-      <c r="F24" s="17" t="n"/>
-      <c r="G24" s="17" t="n"/>
-      <c r="H24" s="17" t="n"/>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="J24" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K24" s="17" t="n"/>
-      <c r="L24" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M24" s="17" t="n"/>
-      <c r="N24" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O24" s="17" t="n"/>
-      <c r="P24" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q24" s="17" t="n"/>
-      <c r="R24" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S24" s="17" t="n"/>
-      <c r="T24" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U24" s="18" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>AUX. CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B25" s="15" t="inlineStr">
-        <is>
-          <t>Gerson Castro</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>Aux. Manutenção / Climatização</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>Diurno par</t>
-        </is>
-      </c>
-      <c r="E25" s="15" t="inlineStr">
-        <is>
-          <t>07:00–19:00</t>
-        </is>
-      </c>
-      <c r="F25" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="G25" s="17" t="n"/>
-      <c r="H25" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I25" s="17" t="n"/>
-      <c r="J25" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K25" s="17" t="n"/>
-      <c r="L25" s="17" t="n"/>
-      <c r="M25" s="17" t="n"/>
-      <c r="N25" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O25" s="17" t="n"/>
-      <c r="P25" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q25" s="17" t="n"/>
-      <c r="R25" s="17" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S25" s="17" t="n"/>
-      <c r="T25" s="17" t="n"/>
-      <c r="U25" s="18" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>AUX. CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Gustavo Rafael Pereira Vargas</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Aux. Manutenção / Climatização</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Diurno ímpar</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>07:00–19:00</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="n"/>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="n"/>
-      <c r="M26" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N26" s="5" t="n"/>
-      <c r="O26" s="5" t="n"/>
-      <c r="P26" s="5" t="n"/>
-      <c r="Q26" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R26" s="5" t="n"/>
-      <c r="S26" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T26" s="5" t="n"/>
-      <c r="U26" s="5" t="inlineStr">
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="n"/>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="n"/>
+      <c r="M26" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N26" s="8" t="n"/>
+      <c r="O26" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P26" s="8" t="n"/>
+      <c r="Q26" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="R26" s="8" t="n"/>
+      <c r="S26" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T26" s="8" t="n"/>
+      <c r="U26" s="9" t="inlineStr">
         <is>
           <t>P</t>
         </is>
@@ -2488,7 +2496,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Victor Hugo Gomes de Araujo</t>
+          <t>Em processo de contratação</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -2498,511 +2506,367 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Noturno par</t>
+          <t>Folguista diurno</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
+          <t>07:00–19:00</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="n"/>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="L27" s="8" t="n"/>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="N27" s="8" t="n"/>
+      <c r="O27" s="8" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="n"/>
+      <c r="Q27" s="8" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="R27" s="8" t="n"/>
+      <c r="S27" s="8" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="T27" s="8" t="n"/>
+      <c r="U27" s="9" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>AUX. CLIMATIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Em processo de contratação</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Aux. Manutenção / Climatização</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Folguista noturno</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
           <t>19:00–07:00</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="n"/>
-      <c r="H27" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="n"/>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="n"/>
-      <c r="L27" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M27" s="8" t="n"/>
-      <c r="N27" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O27" s="8" t="n"/>
-      <c r="P27" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q27" s="8" t="n"/>
-      <c r="R27" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S27" s="8" t="n"/>
-      <c r="T27" s="8" t="n"/>
-      <c r="U27" s="9" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>AUX. CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Jeferson Leandro Nardy Andrade</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Aux. Manutenção / Climatização</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>Noturno ímpar</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>19:00–07:00</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H28" s="8" t="n"/>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J28" s="8" t="n"/>
-      <c r="K28" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L28" s="8" t="n"/>
-      <c r="M28" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N28" s="8" t="n"/>
-      <c r="O28" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P28" s="8" t="n"/>
-      <c r="Q28" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R28" s="8" t="n"/>
-      <c r="S28" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T28" s="8" t="n"/>
-      <c r="U28" s="9" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="n"/>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="n"/>
+      <c r="M28" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="n"/>
+      <c r="O28" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="P28" s="12" t="n"/>
+      <c r="Q28" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="R28" s="12" t="n"/>
+      <c r="S28" s="12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="T28" s="12" t="n"/>
+      <c r="U28" s="13" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>AUX. CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Em processo de contratação</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Aux. Manutenção / Climatização</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Folguista diurno</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>07:00–19:00</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="n"/>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="n"/>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="n"/>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="L29" s="8" t="n"/>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="N29" s="8" t="n"/>
-      <c r="O29" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="P29" s="8" t="n"/>
-      <c r="Q29" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="R29" s="8" t="n"/>
-      <c r="S29" s="8" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="T29" s="8" t="n"/>
-      <c r="U29" s="9" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>COMERCIAL</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>William de Souza Lobo</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Supervisor de Manutenção</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Regime comercial</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>08:00–17:00</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L29" s="12" t="n"/>
+      <c r="M29" s="12" t="n"/>
+      <c r="N29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="R29" s="12" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S29" s="12" t="n"/>
+      <c r="T29" s="12" t="n"/>
+      <c r="U29" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>AUX. CLIMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Em processo de contratação</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Aux. Manutenção / Climatização</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>Folguista noturno</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>19:00–07:00</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="H30" s="12" t="n"/>
-      <c r="I30" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="J30" s="12" t="n"/>
-      <c r="K30" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="L30" s="12" t="n"/>
-      <c r="M30" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="n"/>
-      <c r="O30" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="P30" s="12" t="n"/>
-      <c r="Q30" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="R30" s="12" t="n"/>
-      <c r="S30" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="T30" s="12" t="n"/>
-      <c r="U30" s="13" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>COMERCIAL</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Osmair Pereira de Freitas</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Aux. Administrativo / Analista de Dados</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Regime comercial</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>08:00–17:00</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="n"/>
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="R30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S30" s="5" t="n"/>
+      <c r="T30" s="5" t="n"/>
+      <c r="U30" s="5" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>COMERCIAL</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>William de Souza Lobo</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Supervisor de Manutenção</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>Regime comercial</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>08:00–17:00</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="n"/>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L31" s="12" t="n"/>
-      <c r="M31" s="12" t="n"/>
-      <c r="N31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R31" s="12" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S31" s="12" t="n"/>
-      <c r="T31" s="12" t="n"/>
-      <c r="U31" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="8" t="n"/>
+      <c r="K31" s="8" t="n"/>
+      <c r="L31" s="8" t="n"/>
+      <c r="M31" s="8" t="n"/>
+      <c r="N31" s="8" t="n"/>
+      <c r="O31" s="8" t="n"/>
+      <c r="P31" s="8" t="n"/>
+      <c r="Q31" s="8" t="n"/>
+      <c r="R31" s="8" t="n"/>
+      <c r="S31" s="8" t="n"/>
+      <c r="T31" s="8" t="n"/>
+      <c r="U31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>COMERCIAL</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Osmair Pereira de Freitas</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Aux. Administrativo / Analista de Dados</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Regime comercial</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>08:00–17:00</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L32" s="5" t="n"/>
-      <c r="M32" s="5" t="n"/>
-      <c r="N32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="R32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S32" s="5" t="n"/>
-      <c r="T32" s="5" t="n"/>
-      <c r="U32" s="5" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+      <c r="A32" s="23" t="n"/>
+      <c r="B32" s="23" t="n"/>
+      <c r="C32" s="23" t="n"/>
+      <c r="D32" s="23" t="n"/>
+      <c r="E32" s="23" t="n"/>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="23" t="n"/>
+      <c r="L32" s="23" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="23" t="n"/>
+      <c r="O32" s="23" t="n"/>
+      <c r="P32" s="23" t="n"/>
+      <c r="Q32" s="23" t="n"/>
+      <c r="R32" s="23" t="n"/>
+      <c r="S32" s="23" t="n"/>
+      <c r="T32" s="23" t="n"/>
+      <c r="U32" s="23" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="8" t="n"/>
-      <c r="G33" s="8" t="n"/>
-      <c r="H33" s="8" t="n"/>
-      <c r="I33" s="8" t="n"/>
-      <c r="J33" s="8" t="n"/>
-      <c r="K33" s="8" t="n"/>
-      <c r="L33" s="8" t="n"/>
-      <c r="M33" s="8" t="n"/>
-      <c r="N33" s="8" t="n"/>
-      <c r="O33" s="8" t="n"/>
-      <c r="P33" s="8" t="n"/>
-      <c r="Q33" s="8" t="n"/>
-      <c r="R33" s="8" t="n"/>
-      <c r="S33" s="8" t="n"/>
-      <c r="T33" s="8" t="n"/>
-      <c r="U33" s="9" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="23" t="n"/>
-      <c r="B34" s="23" t="n"/>
-      <c r="C34" s="23" t="n"/>
-      <c r="D34" s="23" t="n"/>
-      <c r="E34" s="23" t="n"/>
-      <c r="F34" s="23" t="n"/>
-      <c r="G34" s="23" t="n"/>
-      <c r="H34" s="23" t="n"/>
-      <c r="I34" s="23" t="n"/>
-      <c r="J34" s="23" t="n"/>
-      <c r="K34" s="23" t="n"/>
-      <c r="L34" s="23" t="n"/>
-      <c r="M34" s="23" t="n"/>
-      <c r="N34" s="23" t="n"/>
-      <c r="O34" s="23" t="n"/>
-      <c r="P34" s="23" t="n"/>
-      <c r="Q34" s="23" t="n"/>
-      <c r="R34" s="23" t="n"/>
-      <c r="S34" s="23" t="n"/>
-      <c r="T34" s="23" t="n"/>
-      <c r="U34" s="23" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="31" t="inlineStr">
+      <c r="A33" s="31" t="inlineStr">
         <is>
           <t>Os dias de presença dos colaboradores já constantes na escala recebida foram preservados, exceto pelas correções formalmente informadas: Carlos Alberto retorna ao diurno par em 16/08; Jeferson Leandro permanece no noturno ímpar, pois suas férias foram prorrogadas para período ainda não informado; Jean Nascimento de Matos foi desligado em 14/08. Osmar integra em 19/08 e assume provisoriamente o noturno par a partir de 20/08; 16 e 18/08 permanecem como cobertura pendente. Célula vazia = descanso/sem expediente; não foi utilizado o código F.</t>
         </is>
       </c>
     </row>
+    <row r="34"/>
+    <row r="35"/>
     <row r="37" ht="42" customHeight="1"/>
   </sheetData>
   <mergeCells count="7">
@@ -3630,7 +3494,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Admissao confirmada em 20/08; folguista diurno impar a partir de 21/08.</t>
+          <t>Milton Gustavo desistiu da vaga e foi retirado da escala.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -3655,7 +3519,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Marcos Lira: folguista diurno impar, admissao confirmada em 21/08. Osmar Silva: noturno par, admissao confirmada em 24/08. Caio Pereira: folguista volante diurno par, admissao confirmada em 20/08.</t>
+          <t>Marcos Lira desistiu da vaga e foi retirado da escala. Osmar Silva: noturno par, admissao confirmada em 24/08. Caio Pereira: folguista volante diurno par, admissao confirmada em 20/08.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">

</xml_diff>